<commit_message>
Daily EOD data and reports for 2026-08-24
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260824.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260824.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.822</v>
+        <v>1.83</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.027</v>
+        <v>0.035</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.50%</t>
+          <t>1.95%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>279095.78</v>
+        <v>280321.23</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>4135.89</v>
+        <v>5361.34</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.395</v>
+        <v>2.38</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.005</v>
+        <v>-0.01</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.21%</t>
+          <t>-0.42%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>167650</v>
+        <v>166600</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>350</v>
+        <v>-700</v>
       </c>
     </row>
     <row r="6">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>67.28</v>
+        <v>67.17</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.12</v>
+        <v>2.01</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.25%</t>
+          <t>3.08%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>744453.2</v>
+        <v>743236.05</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>23457.8</v>
+        <v>22240.65</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>155.12</v>
+        <v>155.04</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-2.87</v>
+        <v>-2.95</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-1.82%</t>
+          <t>-1.87%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>170.745</v>
+        <v>170.12</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>2.445</v>
+        <v>1.82</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.45%</t>
+          <t>1.08%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>682980</v>
+        <v>680480</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>9780</v>
+        <v>7280</v>
       </c>
     </row>
     <row r="12">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.1</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>33.63</v>
+        <v>33.59</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.2</v>
+        <v>-0.24</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.59%</t>
+          <t>-0.71%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>33.54</v>
+        <v>33.51</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.24</v>
+        <v>-0.27</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-0.71%</t>
+          <t>-0.80%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>43199.52</v>
+        <v>43160.88</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-309.12</v>
+        <v>-347.76</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1934196.09</v>
+        <v>1931215.75</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-31711.29</v>
+        <v>-34691.63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>